<commit_message>
chore: update funding tracker
</commit_message>
<xml_diff>
--- a/site/funding-tracker.xlsx
+++ b/site/funding-tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R0c8ccae558f5444f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="Rabd730b84bea4703"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="Rba3a3a15413a4830"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中国公司" sheetId="1" r:id="R5f166eea3e264e13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全球公司" sheetId="2" r:id="Rd5906e8889d64ccc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行日志" sheetId="3" r:id="R6eba3617dbf84fd7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -712,232 +712,226 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>先博生物</x:v>
+        <x:v>芯光界</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>创新药 / 细胞治疗</x:v>
+        <x:v>光互连 / 硅光通信</x:v>
       </x:c>
       <x:c r="C12" s="13" t="n">
-        <x:v>46265.333333333336</x:v>
+        <x:v>46266.333333333336</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>近4亿元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>天使+轮</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G12" s="14"/>
       <x:c r="H12" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>中国证券报·中证网</x:v>
       </x:c>
       <x:c r="I12" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%85%88%E5%8D%9A%E7%94%9F%E7%89%A9%20%E8%BF%914%E4%BA%BF%E5%85%83%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://www.cs.com.cn/tzjj/01/2026/09/02/detail_2026090210036492.html</x:v>
       </x:c>
       <x:c r="J12" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K12" s="12" t="str">
-        <x:v>媒体与官网交叉核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L12" s="12" t="str">
-        <x:v>先博生物（Simnova Bio）是一家创新药和细胞治疗公司，重点推进实体瘤及免疫相关疾病方向的候选产品研发。公司围绕细胞治疗、基因工程和转化医学平台建设管线，服务临床未满足需求。</x:v>
+        <x:v>芯光界面向 AI 算力集群和高速通信场景研发硅光互连与光电融合产品。公司聚焦低功耗、高带宽、可规模化部署的光互连方案，服务数据中心、智算中心和下一代网络基础设施。</x:v>
       </x:c>
       <x:c r="M12" s="12" t="str">
-        <x:v>https://www.simnovabio.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N12" s="12" t="str">
-        <x:v>官网联系页：https://www.simnovabio.com/cn/contact-us</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>灵初智能</x:v>
+        <x:v>先博生物</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
-        <x:v>具身智能 / 机器人</x:v>
+        <x:v>创新药 / 细胞治疗</x:v>
       </x:c>
       <x:c r="C13" s="13" t="n">
-        <x:v>46261.333333333336</x:v>
+        <x:v>46265.333333333336</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>过亿美元</x:v>
+        <x:v>近4亿元人民币</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
         <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="G13" s="14" t="n">
-        <x:v>72000</x:v>
-      </x:c>
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G13" s="14"/>
       <x:c r="H13" s="12" t="str">
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I13" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%81%B5%E5%88%9D%E6%99%BA%E8%83%BD%20%E8%BF%87%E4%BA%BF%E7%BE%8E%E5%85%83%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E5%85%88%E5%8D%9A%E7%94%9F%E7%89%A9%20%E8%BF%914%E4%BA%BF%E5%85%83%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J13" s="15" t="n">
         <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K13" s="12" t="str">
-        <x:v>媒体核验；官网待交叉确认</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L13" s="12" t="str">
-        <x:v>灵初智能专注具身智能与机器人基础模型，研发面向真实物理世界操作的感知、决策和控制系统。公司目标是通过大模型、仿真训练和机器人本体能力结合，提升通用机器人在工业、服务和家庭场景中的可用性。</x:v>
+        <x:v>先博生物（Simnova Bio）是一家创新药和细胞治疗公司，重点推进实体瘤及免疫相关疾病方向的候选产品研发。公司围绕细胞治疗、基因工程和转化医学平台建设管线，服务临床未满足需求。</x:v>
       </x:c>
       <x:c r="M13" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.simnovabio.com/</x:v>
       </x:c>
       <x:c r="N13" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网联系页：https://www.simnovabio.com/cn/contact-us</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
-        <x:v>蜂巢互联</x:v>
+        <x:v>沐创集成电路</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>工业软件 / 物理 AI 仿真</x:v>
+        <x:v>智能网卡 / 高速互联芯片</x:v>
       </x:c>
       <x:c r="C14" s="13" t="n">
-        <x:v>46260.333333333336</x:v>
+        <x:v>46264.333333333336</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>12亿元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
-        <x:v>战略融资</x:v>
+        <x:v>B 轮</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G14" s="14" t="n">
-        <x:v>120000</x:v>
-      </x:c>
+      <x:c r="G14" s="14"/>
       <x:c r="H14" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I14" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E8%9C%82%E5%B7%A2%E4%BA%92%E8%81%94%2012%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84%20%E7%89%A9%E7%90%86AI%E4%BB%BF%E7%9C%9F%E5%BC%95%E6%93%8E&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J14" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K14" s="12" t="str">
         <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L14" s="12" t="str">
-        <x:v>蜂巢互联提供工业软件、数字孪生和物理 AI 仿真能力，面向制造业复杂设备和产线构建虚实融合平台。公司通过仿真引擎、工业互联网和数据模型，支持研发验证、生产优化和智能运维场景。</x:v>
+        <x:v>沐创集成电路专注智能网卡、DPU 和高速互联芯片研发，面向数据中心、云计算和智算基础设施提供网络与数据处理芯片。公司产品服务高吞吐、低延迟的数据传输和计算卸载场景。</x:v>
       </x:c>
       <x:c r="M14" s="12" t="str">
-        <x:v>https://www.vbullet.com/</x:v>
+        <x:v>https://www.mucse.com/</x:v>
       </x:c>
       <x:c r="N14" s="12" t="str">
-        <x:v>官网联系页：https://www.vbullet.com/</x:v>
+        <x:v>官网联系页：https://www.mucse.com/contact.html</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>小鹏机器人</x:v>
+        <x:v>研微半导体</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>人形机器人 / 具身智能</x:v>
+        <x:v>半导体设备 / 薄膜沉积</x:v>
       </x:c>
       <x:c r="C15" s="13" t="n">
-        <x:v>46258.333333333336</x:v>
+        <x:v>46264.333333333336</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>超9亿美元</x:v>
+        <x:v>近15亿元人民币</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>首轮融资</x:v>
+        <x:v>B 轮</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="G15" s="14" t="n">
-        <x:v>648000</x:v>
-      </x:c>
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G15" s="14"/>
       <x:c r="H15" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I15" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%B0%8F%E9%B9%8F%E6%9C%BA%E5%99%A8%E4%BA%BA%20%E8%B6%859%E4%BA%BF%E7%BE%8E%E5%85%83%20%E9%A6%96%E8%BD%AE%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J15" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K15" s="12" t="str">
-        <x:v>媒体交叉核验</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L15" s="12" t="str">
-        <x:v>小鹏机器人是小鹏体系内面向人形机器人和具身智能方向的业务，公开展示过 IRON 等机器人产品。其研发围绕机器人本体、运动控制、环境感知和智能交互展开，目标是将智能汽车相关技术能力延伸到机器人场景。</x:v>
+        <x:v>研微半导体聚焦半导体薄膜沉积设备和关键制程装备研发，服务集成电路、先进封装和泛半导体制造。公司围绕国产半导体设备替代、工艺适配和产线交付推进产业化。</x:v>
       </x:c>
       <x:c r="M15" s="12" t="str">
-        <x:v>https://www.xpeng.com/</x:v>
+        <x:v>https://www.psrsemi.com/</x:v>
       </x:c>
       <x:c r="N15" s="12" t="str">
-        <x:v>官网联系页：https://www.xpeng.com/contact</x:v>
+        <x:v>官网联系页：https://www.psrsemi.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>枢途科技</x:v>
+        <x:v>迈步机器人</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>AGI Infra / AI 数据基础设施</x:v>
+        <x:v>康复机器人 / 外骨骼</x:v>
       </x:c>
       <x:c r="C16" s="13" t="n">
-        <x:v>46258.333333333336</x:v>
+        <x:v>46264.333333333336</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>近亿元人民币</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>连续两轮融资</x:v>
+        <x:v>战略融资</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G16" s="14"/>
       <x:c r="H16" s="12" t="str">
-        <x:v>36氪</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I16" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%9E%A2%E9%80%94%E7%A7%91%E6%8A%80%20%E8%BF%9E%E7%BB%AD%E5%AE%8C%E6%88%90%E4%B8%A4%E8%BD%AE%E8%9E%8D%E8%B5%84%202026&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J16" s="15" t="n">
-        <x:v>46272.748611111114</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K16" s="12" t="str">
-        <x:v>媒体核验；官网待交叉确认</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L16" s="12" t="str">
-        <x:v>枢途科技聚焦 AGI Infra 与 AI 数据基础设施，面向大模型训练、智能体开发和企业 AI 应用提供底层数据与工程平台。公司强调数据流、知识组织和模型应用之间的连接能力，帮助团队更高效地构建可落地的智能系统。</x:v>
+        <x:v>迈步机器人是一家康复机器人和外骨骼设备企业，产品覆盖下肢康复训练、步态训练和智能辅助行走等方向。公司面向医院、康复中心和家庭康复场景，结合机器人控制、传感和康复医学提升训练效率。</x:v>
       </x:c>
       <x:c r="M16" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.milebot.com/</x:v>
       </x:c>
       <x:c r="N16" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网联系页：https://www.milebot.com/contact.html</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>嘉腾机器人</x:v>
+        <x:v>屹艮科技</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>工业具身智能 / AGV / AMR</x:v>
+        <x:v>AI for Science / 电池设计自动化</x:v>
       </x:c>
       <x:c r="C17" s="13" t="n">
-        <x:v>46252.333333333336</x:v>
+        <x:v>46264.333333333336</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>亿元级人民币</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
         <x:v>战略融资</x:v>
@@ -947,39 +941,39 @@
       </x:c>
       <x:c r="G17" s="14"/>
       <x:c r="H17" s="12" t="str">
-        <x:v>21世纪经济报道</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I17" s="16" t="str">
-        <x:v>https://m.21jingji.com/article/20260818/herald/09ad8c401fbb711d0cd6717d4988613c.html</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J17" s="15" t="n">
-        <x:v>46253.82167824074</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K17" s="12" t="str">
-        <x:v>媒体交叉核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L17" s="12" t="str">
-        <x:v>嘉腾机器人专注工业自动化解决方案与机器人研发制造，重点布局 AGV、AMR 及具身智能移动底盘等产品。公司面向制造、仓储、物流与工业搬运场景，强调规模化交付和全球化应用能力。</x:v>
+        <x:v>屹艮科技面向电池材料研发和电池设计自动化建设 AI for Science 平台，支持材料筛选、配方设计和性能预测。公司将机器学习、实验数据和多尺度仿真结合，服务新能源电池研发效率提升。</x:v>
       </x:c>
       <x:c r="M17" s="12" t="str">
-        <x:v>https://www.jtrobots.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N17" s="12" t="str">
-        <x:v>总机电话：400-830-1028；商务邮箱：marketing@jtrobots.com；官网联系页：https://www.jtrobots.com/address</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>灵锶智能</x:v>
+        <x:v>中数睿智</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>四足机器人 / 人形机器人</x:v>
+        <x:v>大模型 / 企业 AI Agent</x:v>
       </x:c>
       <x:c r="C18" s="13" t="n">
-        <x:v>46252.333333333336</x:v>
+        <x:v>46264.333333333336</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
-        <x:v>7000万元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
         <x:v>战略融资</x:v>
@@ -987,237 +981,235 @@
       <x:c r="F18" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G18" s="14" t="n">
-        <x:v>7000</x:v>
-      </x:c>
+      <x:c r="G18" s="14"/>
       <x:c r="H18" s="12" t="str">
-        <x:v>新浪科技</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I18" s="16" t="str">
-        <x:v>https://finance.sina.com.cn/tech/roll/2026-08-18/doc-inintpin8618761.shtml</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J18" s="15" t="n">
-        <x:v>46253.82167824074</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K18" s="12" t="str">
-        <x:v>媒体交叉核验</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L18" s="12" t="str">
-        <x:v>灵锶智能聚焦四足机器人与人形 AI 机器人研发，产品面向电力巡检、应急救援、工厂巡检等复杂工业场景。公司强调重载、长续航和复杂地形适应能力，并在广东机器人产业链中持续推进产品化。</x:v>
+        <x:v>中数睿智聚焦企业级大模型和 AI Agent 应用，推出语思等面向行业知识、办公协同和智能决策的产品体系。公司服务政府、央国企和大型组织的数字化与智能化升级场景。</x:v>
       </x:c>
       <x:c r="M18" s="12" t="str">
-        <x:v>https://www.gdlinxai.com/</x:v>
+        <x:v>https://www.zhongshuruizhi.com/</x:v>
       </x:c>
       <x:c r="N18" s="12" t="str">
-        <x:v>电话：17710125211；邮箱：info@linxai-tech.com；官网联系页：https://www.gdlinxai.com/h-col-109.html</x:v>
+        <x:v>官网联系页：https://www.zhongshuruizhi.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>安澜德健</x:v>
+        <x:v>星邑空间</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
-        <x:v>医疗器械 / 心室辅助装置</x:v>
+        <x:v>商业航天 / 卫星测运控</x:v>
       </x:c>
       <x:c r="C19" s="13" t="n">
-        <x:v>46252.333333333336</x:v>
+        <x:v>46264.333333333336</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
-        <x:v>近亿元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>A 轮增资扩股</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G19" s="14"/>
       <x:c r="H19" s="12" t="str">
-        <x:v>启明创投</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I19" s="16" t="str">
-        <x:v>https://www.qimingvc.com/cn/news/%E5%90%AF%E6%98%8E%E6%98%9F-%E5%AE%89%E6%BE%9C%E5%BE%B7%E5%81%A5%E5%AE%8C%E6%88%90%E8%BF%91%E4%BA%BF%E5%85%83a%E8%BD%AE%E8%9E%8D%E8%B5%84%EF%BC%8C%E5%90%AF%E6%98%8E%E5%88%9B%E6%8A%95%E7%8B%AC%E5%AE%B6%E6%8A%95%E8%B5%84</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J19" s="15" t="n">
-        <x:v>46253.82167824074</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K19" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L19" s="12" t="str">
-        <x:v>安澜德健（Enginprime Medical）专注经皮心室辅助装置（pVAD）研发，核心产品为 OpusOne™。公司围绕更小尺寸、更高流量的心室辅助系统推进中国注册临床试验与海外早期临床申报。</x:v>
+        <x:v>星邑空间从事商业航天测运控、卫星数据服务和空间信息基础设施建设，面向卫星运营、遥感应用和低轨星座服务提供能力。公司围绕地面站网络、测控调度和空间数据应用推进商业化。</x:v>
       </x:c>
       <x:c r="M19" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.xingyispace.com/</x:v>
       </x:c>
       <x:c r="N19" s="12" t="str">
-        <x:v>媒体邮箱：media@enginprime.com；投资者联系：info@voyagerscap.com</x:v>
+        <x:v>官网联系页：https://www.xingyispace.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
-        <x:v>亿兰科</x:v>
+        <x:v>瞬适科技</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
-        <x:v>高端分析仪器 / 质谱仪</x:v>
+        <x:v>具身智能 / 物理 AI 数据基础设施</x:v>
       </x:c>
       <x:c r="C20" s="13" t="n">
-        <x:v>46245.333333333336</x:v>
+        <x:v>46262.333333333336</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>千万美元</x:v>
       </x:c>
       <x:c r="E20" s="12" t="str">
-        <x:v>Pre-A 轮</x:v>
+        <x:v>种子轮</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="G20" s="14"/>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G20" s="14" t="n">
+        <x:v>7200</x:v>
+      </x:c>
       <x:c r="H20" s="12" t="str">
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I20" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567473.shtml</x:v>
+        <x:v>https://news.pedaily.cn/202608/568250.shtml</x:v>
       </x:c>
       <x:c r="J20" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K20" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L20" s="12" t="str">
-        <x:v>亿兰科专注工商业模块化光储系统和电力电子设备，围绕 PCS、混合逆变器、光储一体机与微电网管理系统开展研发和交付。公司产品服务工商业储能、分布式光伏和海外终端市场。</x:v>
+        <x:v>瞬适科技（InstAdapt）聚焦具身智能与物理 AI 数据基础设施，提供真实物理世界数据采集、标注、训练与评测相关能力。公司面向机器人、自动驾驶和空间智能等场景，帮助模型更快适应动态环境。</x:v>
       </x:c>
       <x:c r="M20" s="12" t="str">
-        <x:v>https://www.elecod.cn/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N20" s="12" t="str">
-        <x:v>电话：0755-23050802；商务邮箱：marketing@elecod.com；人力邮箱：hr@elecod.com；官网联系页：https://www.elecod.cn/aboutus.html。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>诺因智能</x:v>
+        <x:v>灵初智能</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
-        <x:v>具身智能 / 消费级机器人</x:v>
+        <x:v>具身智能 / 机器人</x:v>
       </x:c>
       <x:c r="C21" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46261.333333333336</x:v>
       </x:c>
       <x:c r="D21" s="12" t="str">
-        <x:v>5 亿元人民币</x:v>
+        <x:v>过亿美元</x:v>
       </x:c>
       <x:c r="E21" s="12" t="str">
-        <x:v>天使++轮</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F21" s="12" t="str">
-        <x:v>CNY</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="G21" s="14" t="n">
-        <x:v>50000</x:v>
+        <x:v>72000</x:v>
       </x:c>
       <x:c r="H21" s="12" t="str">
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I21" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567457.shtml</x:v>
+        <x:v>https://news.google.com/search?q=%E7%81%B5%E5%88%9D%E6%99%BA%E8%83%BD%20%E8%BF%87%E4%BA%BF%E7%BE%8E%E5%85%83%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J21" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K21" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L21" s="12" t="str">
-        <x:v>诺因智能聚焦家庭场景具身智能，围绕折叠双臂机器人及相关感知、执行和交互系统推进产品研发。公司目标是让机器人进入真实家庭环境，承担陪伴互动、整理和基础协作等任务。</x:v>
+        <x:v>灵初智能专注具身智能与机器人基础模型，研发面向真实物理世界操作的感知、决策和控制系统。公司目标是通过大模型、仿真训练和机器人本体能力结合，提升通用机器人在工业、服务和家庭场景中的可用性。</x:v>
       </x:c>
       <x:c r="M21" s="12" t="str">
-        <x:v>https://knowinai.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N21" s="12" t="str">
-        <x:v>招聘邮箱：HR@knowin.ai；联系电话：17610340223；媒介合作：media@knowin.ai；官方联系页：https://knowinai.com/。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
-        <x:v>星环聚能</x:v>
+        <x:v>晰见科技</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
-        <x:v>可控聚变 / 清洁能源</x:v>
+        <x:v>类脑视觉芯片 / 物理 AI</x:v>
       </x:c>
       <x:c r="C22" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46261.333333333336</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>8.8 亿元人民币</x:v>
+        <x:v>近5亿元人民币</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>A++ 轮</x:v>
+        <x:v>连续3轮融资</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G22" s="14" t="n">
-        <x:v>88000</x:v>
-      </x:c>
+      <x:c r="G22" s="14"/>
       <x:c r="H22" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>新浪财经 / 投资界</x:v>
       </x:c>
       <x:c r="I22" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567446.shtml</x:v>
+        <x:v>https://finance.sina.com.cn/jjxw/2026-08-27/doc-iniptnuz5849968.shtml</x:v>
       </x:c>
       <x:c r="J22" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K22" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体与公开官网信息交叉核验</x:v>
       </x:c>
       <x:c r="L22" s="12" t="str">
-        <x:v>星环聚能专注可控核聚变相关技术和工程化系统，推动聚变能装备研发及商业化路径。公司面向清洁能源、长期稳定供能和能源转型场景，持续扩展实验和产业化能力。</x:v>
+        <x:v>晰见科技围绕类脑视觉芯片和物理 AI 计算架构开展研发，产品面向低功耗视觉感知、机器人和边缘智能场景。公司试图通过传感、计算和算法协同提升机器在真实环境中的视觉处理效率。</x:v>
       </x:c>
       <x:c r="M22" s="12" t="str">
-        <x:v>https://startorus.cn/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N22" s="12" t="str">
-        <x:v>电话：029-86041002；邮箱：business@startorus.cn；公司地址：上海市嘉定区澄浏公路52号39幢2楼JT109869室；官网联系页：https://startorus.cn/。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="12" t="str">
-        <x:v>奇算光启</x:v>
+        <x:v>艾联纳医药</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
-        <x:v>AI 光计算芯片</x:v>
+        <x:v>创新药 / 小分子药物</x:v>
       </x:c>
       <x:c r="C23" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46261.333333333336</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>超1亿元人民币</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>天使轮及天使+轮</x:v>
+        <x:v>Seed+ 轮</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G23" s="14"/>
       <x:c r="H23" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>大河财立方</x:v>
       </x:c>
       <x:c r="I23" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567453.shtml</x:v>
+        <x:v>https://m.sohu.com/a/1068278269_120109837?scm=10001.325_13-325_13.0.0-0-0-0-0.5_1334</x:v>
       </x:c>
       <x:c r="J23" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K23" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体交叉核验；官网待确认</x:v>
       </x:c>
       <x:c r="L23" s="12" t="str">
-        <x:v>奇算光启专注 AI 光计算芯片和光计算系统研发，试图用全光计算与集成光子技术突破传统电子芯片能效瓶颈。公司面向大模型和高性能计算底座，强调算力密度、功耗和系统扩展能力。</x:v>
+        <x:v>艾联纳医药是一家创新药研发企业，围绕小分子药物发现和疾病靶点验证推进早期管线。公司重点建设药物设计、转化研究和临床前开发能力，服务肿瘤、免疫或其他高未满足需求疾病方向。</x:v>
       </x:c>
       <x:c r="M23" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1228,80 +1220,82 @@
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="12" t="str">
-        <x:v>深度细胞</x:v>
+        <x:v>蜂巢互联</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>AI 医疗 / 单细胞分析</x:v>
+        <x:v>工业软件 / 物理 AI 仿真</x:v>
       </x:c>
       <x:c r="C24" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46260.333333333336</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>近亿元人民币</x:v>
+        <x:v>12亿元人民币</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
-        <x:v>种子轮</x:v>
+        <x:v>战略融资</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G24" s="14"/>
+      <x:c r="G24" s="14" t="n">
+        <x:v>120000</x:v>
+      </x:c>
       <x:c r="H24" s="12" t="str">
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I24" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567451.shtml</x:v>
+        <x:v>https://news.google.com/search?q=%E8%9C%82%E5%B7%A2%E4%BA%92%E8%81%94%2012%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84%20%E7%89%A9%E7%90%86AI%E4%BB%BF%E7%9C%9F%E5%BC%95%E6%93%8E&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J24" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K24" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L24" s="12" t="str">
-        <x:v>深度细胞聚焦 AI 制药与虚拟细胞建模，围绕单细胞分析、疾病机理和药物研发加速构建算法平台。公司目标是把细胞级计算能力用于新药发现和生物医学研究。</x:v>
+        <x:v>蜂巢互联提供工业软件、数字孪生和物理 AI 仿真能力，面向制造业复杂设备和产线构建虚实融合平台。公司通过仿真引擎、工业互联网和数据模型，支持研发验证、生产优化和智能运维场景。</x:v>
       </x:c>
       <x:c r="M24" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://www.vbullet.com/</x:v>
       </x:c>
       <x:c r="N24" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>官网联系页：https://www.vbullet.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="12" t="str">
-        <x:v>橡木果机器人</x:v>
+        <x:v>原力引擎</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
-        <x:v>具身智能 / 人形机器人</x:v>
+        <x:v>AI for Engineering / 生成式仿真</x:v>
       </x:c>
       <x:c r="C25" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46260.333333333336</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>近5000万元人民币</x:v>
       </x:c>
       <x:c r="E25" s="12" t="str">
-        <x:v>天使轮</x:v>
+        <x:v>天使+轮</x:v>
       </x:c>
       <x:c r="F25" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G25" s="14"/>
       <x:c r="H25" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>新浪财经</x:v>
       </x:c>
       <x:c r="I25" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567448.shtml</x:v>
+        <x:v>https://finance.sina.cn/2026-08-26/detail-inipqwax2358348.d.html</x:v>
       </x:c>
       <x:c r="J25" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K25" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L25" s="12" t="str">
-        <x:v>橡木果机器人专注通用具身操作，围绕触觉感知、操作基座模型和机器人执行能力构建底层技术栈。公司强调自下而上的“本能驱动”路线，目标是让机器人在真实物理环境中稳定完成操作任务。</x:v>
+        <x:v>原力引擎聚焦 AI for Engineering 和生成式仿真，面向工程研发提供仿真建模、设计探索和智能优化工具。公司希望用大模型与数值仿真结合，提升工业研发、装备设计和复杂系统工程效率。</x:v>
       </x:c>
       <x:c r="M25" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1312,504 +1306,508 @@
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="12" t="str">
-        <x:v>Noiz AI</x:v>
+        <x:v>赛科动力</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
-        <x:v>AI 语音 / 视听内容生成</x:v>
+        <x:v>固态电池</x:v>
       </x:c>
       <x:c r="C26" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46260.333333333336</x:v>
       </x:c>
       <x:c r="D26" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E26" s="12" t="str">
-        <x:v>种子轮</x:v>
+        <x:v>股权融资</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G26" s="14"/>
       <x:c r="H26" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I26" s="16" t="str">
-        <x:v>https://news.pedaily.cn/202608/567447.shtml</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J26" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K26" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L26" s="12" t="str">
-        <x:v>Noiz AI 提供文本转语音、声音克隆和语音设计能力，面向内容创作、配音、本地化和开发者 API 场景。其产品强调情感控制、低延迟生成和多语言语音输出，服务全球化音频工作流。</x:v>
+        <x:v>赛科动力专注固态电池技术研发与产业化，围绕高安全、高能量密度电池材料、工艺和电芯产品推进量产。公司面向新能源汽车、低空飞行器、储能和消费电子等应用场景。</x:v>
       </x:c>
       <x:c r="M26" s="12" t="str">
-        <x:v>https://noiz.ai/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N26" s="12" t="str">
-        <x:v>邮箱：contact@noiz.ai；官网联系页：https://noiz.ai/。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="12" t="str">
-        <x:v>飞声</x:v>
+        <x:v>简智机器人</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
-        <x:v>AI 助听器 / 医疗器械</x:v>
+        <x:v>具身智能 / 数据基础设施</x:v>
       </x:c>
       <x:c r="C27" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46260.333333333336</x:v>
       </x:c>
       <x:c r="D27" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>未披露</x:v>
       </x:c>
       <x:c r="E27" s="12" t="str">
-        <x:v>天使轮</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F27" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G27" s="14"/>
       <x:c r="H27" s="12" t="str">
-        <x:v>36氪</x:v>
+        <x:v>园区世界投融资周报</x:v>
       </x:c>
       <x:c r="I27" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E9%A3%9E%E5%A3%B0%20AI%20%E5%8A%A9%E5%90%AC%E5%99%A8%20%E5%A4%A9%E4%BD%BF%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://www.parkworld.net/post/8df067aa2cc23f2</x:v>
       </x:c>
       <x:c r="J27" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K27" s="12" t="str">
-        <x:v>媒体与官网交叉核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L27" s="12" t="str">
-        <x:v>飞声专注 AI 助听器与听力辅助产品，结合声学处理、语音增强和智能交互能力改善听障场景的佩戴体验。公司面向消费级与医疗级场景推进产品化，强调清晰拾音、降噪和更自然的听觉补偿。</x:v>
+        <x:v>简智机器人围绕具身智能数据基础设施和机器人数据闭环构建平台能力，支持机器人模型训练、评测与部署。公司面向通用机器人、工业机器人和智能体开发场景，强调高质量数据和模型迭代效率。</x:v>
       </x:c>
       <x:c r="M27" s="12" t="str">
-        <x:v>https://www.flysounds.cn/zh/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N27" s="12" t="str">
-        <x:v>电话：15828225541；商务邮箱：jory@flysounds.com；地址：深圳市龙华区龙华街道清湖社区大和路356号金鼎盛科创园A栋18楼。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="12" t="str">
-        <x:v>霍德生物</x:v>
+        <x:v>小鹏机器人</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>细胞治疗 / 生物技术</x:v>
+        <x:v>人形机器人 / 具身智能</x:v>
       </x:c>
       <x:c r="C28" s="13" t="n">
-        <x:v>46244.333333333336</x:v>
+        <x:v>46258.333333333336</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
-        <x:v>近 2 亿元人民币</x:v>
+        <x:v>超9亿美元</x:v>
       </x:c>
       <x:c r="E28" s="12" t="str">
-        <x:v>C 轮首关</x:v>
+        <x:v>首轮融资</x:v>
       </x:c>
       <x:c r="F28" s="12" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="G28" s="14"/>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G28" s="14" t="n">
+        <x:v>648000</x:v>
+      </x:c>
       <x:c r="H28" s="12" t="str">
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I28" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E9%9C%8D%E5%BE%B7%E7%94%9F%E7%89%A9%20%E8%BF%91%202%20%E4%BA%BF%E5%85%83%20C%E8%BD%AE%20%E9%A6%96%E5%85%B3&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E5%B0%8F%E9%B9%8F%E6%9C%BA%E5%99%A8%E4%BA%BA%20%E8%B6%859%E4%BA%BF%E7%BE%8E%E5%85%83%20%E9%A6%96%E8%BD%AE%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J28" s="15" t="n">
-        <x:v>46245.44097222222</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K28" s="12" t="str">
-        <x:v>媒体与公开工商信息交叉核验</x:v>
+        <x:v>媒体交叉核验</x:v>
       </x:c>
       <x:c r="L28" s="12" t="str">
-        <x:v>霍德生物工程有限公司聚焦细胞治疗和再生医学相关技术与产品，围绕研发、工艺和临床转化推进管线建设。公司在公开页面中长期披露研发动态与产品进展，面向生物医药产业化需求。</x:v>
+        <x:v>小鹏机器人是小鹏体系内面向人形机器人和具身智能方向的业务，公开展示过 IRON 等机器人产品。其研发围绕机器人本体、运动控制、环境感知和智能交互展开，目标是将智能汽车相关技术能力延伸到机器人场景。</x:v>
       </x:c>
       <x:c r="M28" s="12" t="str">
-        <x:v>https://www.hopstem.com/</x:v>
+        <x:v>https://www.xpeng.com/</x:v>
       </x:c>
       <x:c r="N28" s="12" t="str">
-        <x:v>电话：0571-88197776；邮箱：info@hopstem.com；官网联系页：https://www.hopstem.com/。</x:v>
+        <x:v>官网联系页：https://www.xpeng.com/contact</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="12" t="str">
-        <x:v>可灵 AI</x:v>
+        <x:v>枢途科技</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>AI 视频大模型</x:v>
+        <x:v>AGI Infra / AI 数据基础设施</x:v>
       </x:c>
       <x:c r="C29" s="13" t="n">
-        <x:v>46241.333333333336</x:v>
+        <x:v>46258.333333333336</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
-        <x:v>近 30 亿美元</x:v>
+        <x:v>未披露</x:v>
       </x:c>
       <x:c r="E29" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>连续两轮融资</x:v>
       </x:c>
       <x:c r="F29" s="12" t="str">
-        <x:v>USD</x:v>
+        <x:v>CNY</x:v>
       </x:c>
       <x:c r="G29" s="14"/>
       <x:c r="H29" s="12" t="str">
-        <x:v>新华网 / 经济参考报</x:v>
+        <x:v>36氪</x:v>
       </x:c>
       <x:c r="I29" s="16" t="str">
-        <x:v>https://www.news.cn/tech/20260807/1605ef446e5045b7ba0ee55245ce731c/c.html</x:v>
+        <x:v>https://news.google.com/search?q=%E6%9E%A2%E9%80%94%E7%A7%91%E6%8A%80%20%E8%BF%9E%E7%BB%AD%E5%AE%8C%E6%88%90%E4%B8%A4%E8%BD%AE%E8%9E%8D%E8%B5%84%202026&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J29" s="15" t="n">
-        <x:v>46242.48541666667</x:v>
+        <x:v>46272.748611111114</x:v>
       </x:c>
       <x:c r="K29" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L29" s="12" t="str">
-        <x:v>可灵 AI 是面向视频生成与创作的 AI 大模型产品，支持文本、图片等输入驱动的视频内容生成和编辑。产品服务广告创意、影视内容、社交媒体和商业化营销等场景，重点提升视频生成的一致性、可控性和创作效率。</x:v>
+        <x:v>枢途科技聚焦 AGI Infra 与 AI 数据基础设施，面向大模型训练、智能体开发和企业 AI 应用提供底层数据与工程平台。公司强调数据流、知识组织和模型应用之间的连接能力，帮助团队更高效地构建可落地的智能系统。</x:v>
       </x:c>
       <x:c r="M29" s="12" t="str">
-        <x:v>https://klingai.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N29" s="12" t="str">
-        <x:v>商务联系：官网联系页</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="12" t="str">
-        <x:v>矩阵起源</x:v>
+        <x:v>中科第五纪</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
-        <x:v>企业级 AI 基础设施</x:v>
+        <x:v>具身智能 / 具身大脑</x:v>
       </x:c>
       <x:c r="C30" s="13" t="n">
-        <x:v>46240.333333333336</x:v>
+        <x:v>46254.333333333336</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>超 1,000 万美元</x:v>
+        <x:v>超10亿元人民币</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>A1、A2 轮</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="G30" s="14" t="n">
-        <x:v>7200</x:v>
-      </x:c>
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G30" s="14"/>
       <x:c r="H30" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>科创板日报 / 东方财富</x:v>
       </x:c>
       <x:c r="I30" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%9F%A9%E9%98%B5%E8%B5%B7%E6%BA%90%20%E8%B6%85%E5%8D%83%E4%B8%87%E7%BE%8E%E5%85%83%20A%E8%BD%AE%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://finance.eastmoney.com/a/202608203847689590.html</x:v>
       </x:c>
       <x:c r="J30" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46272.77361111111</x:v>
       </x:c>
       <x:c r="K30" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体核验；官网待交叉确认</x:v>
       </x:c>
       <x:c r="L30" s="12" t="str">
-        <x:v>矩阵起源专注 AI 原生数据基础设施，提供多模态数据处理、数据库与企业级 AI 数据底座产品及解决方案。其产品面向企业在结构化、非结构化和向量数据之间建立统一的数据管理与计算能力，为模型训练、知识检索和 AI 应用部署提供底层支撑。</x:v>
+        <x:v>中科第五纪专注具身智能和具身大脑技术，围绕机器人感知、决策、动作生成和世界模型构建基础能力。公司面向通用机器人、工业智能和真实世界交互场景推进产品化。</x:v>
       </x:c>
       <x:c r="M30" s="12" t="str">
-        <x:v>https://matrixorigin.cn/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N30" s="12" t="str">
-        <x:v>商务邮箱：contact@matrixorigin.cn。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="12" t="str">
-        <x:v>为光能源</x:v>
+        <x:v>嘉腾机器人</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
-        <x:v>电力电子 / 固态变压器</x:v>
+        <x:v>工业具身智能 / AGV / AMR</x:v>
       </x:c>
       <x:c r="C31" s="13" t="n">
-        <x:v>46240.333333333336</x:v>
+        <x:v>46252.333333333336</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
-        <x:v>B 轮</x:v>
+        <x:v>战略融资</x:v>
       </x:c>
       <x:c r="F31" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G31" s="14"/>
       <x:c r="H31" s="12" t="str">
-        <x:v>中国网</x:v>
+        <x:v>21世纪经济报道</x:v>
       </x:c>
       <x:c r="I31" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E4%B8%BA%E5%85%89%E8%83%BD%E6%BA%90%20B%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://m.21jingji.com/article/20260818/herald/09ad8c401fbb711d0cd6717d4988613c.html</x:v>
       </x:c>
       <x:c r="J31" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46253.82167824074</x:v>
       </x:c>
       <x:c r="K31" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体交叉核验</x:v>
       </x:c>
       <x:c r="L31" s="12" t="str">
-        <x:v>西安为光能源科技有限公司聚焦固态变压器（SST）等新型电力电子装备及能源互联网解决方案。公司瞄准算力中心、电动交通、新型配网和储能等高功率密度场景，通过电能变换、控制和系统集成提升供配电效率与灵活性。</x:v>
+        <x:v>嘉腾机器人专注工业自动化解决方案与机器人研发制造，重点布局 AGV、AMR 及具身智能移动底盘等产品。公司面向制造、仓储、物流与工业搬运场景，强调规模化交付和全球化应用能力。</x:v>
       </x:c>
       <x:c r="M31" s="12" t="str">
-        <x:v>https://www.weiguangenergy.com/</x:v>
+        <x:v>https://www.jtrobots.com/</x:v>
       </x:c>
       <x:c r="N31" s="12" t="str">
-        <x:v>服务热线：400-868-6988；商务邮箱（官网公开）：wangjuan0509@foxmail.com；地址：陕西省西安市高新区毕原二路3号先导院南区5-6号楼；公众号：WGenergy；在线留言：官网联系页。</x:v>
+        <x:v>总机电话：400-830-1028；商务邮箱：marketing@jtrobots.com；官网联系页：https://www.jtrobots.com/address</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="12" t="str">
-        <x:v>飞捷科思</x:v>
+        <x:v>灵锶智能</x:v>
       </x:c>
       <x:c r="B32" s="12" t="str">
-        <x:v>半导体</x:v>
+        <x:v>四足机器人 / 人形机器人</x:v>
       </x:c>
       <x:c r="C32" s="13" t="n">
-        <x:v>46240.333333333336</x:v>
+        <x:v>46252.333333333336</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>7000万元人民币</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
-        <x:v>A1 轮</x:v>
+        <x:v>战略融资</x:v>
       </x:c>
       <x:c r="F32" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G32" s="14"/>
+      <x:c r="G32" s="14" t="n">
+        <x:v>7000</x:v>
+      </x:c>
       <x:c r="H32" s="12" t="str">
-        <x:v>观点网</x:v>
+        <x:v>新浪科技</x:v>
       </x:c>
       <x:c r="I32" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E9%A3%9E%E6%8D%B7%E7%A7%91%E6%80%9D%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://finance.sina.com.cn/tech/roll/2026-08-18/doc-inintpin8618761.shtml</x:v>
       </x:c>
       <x:c r="J32" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46253.82167824074</x:v>
       </x:c>
       <x:c r="K32" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体交叉核验</x:v>
       </x:c>
       <x:c r="L32" s="12" t="str">
-        <x:v>飞捷科思以高精度实时物理仿真引擎为核心，研发面向具身智能和人形机器人的物理智能技术与产品。其能力重点在于让机器人在虚拟环境中完成动力学、接触和运动策略验证，以缩短从算法训练到真实机器部署的迭代周期。</x:v>
+        <x:v>灵锶智能聚焦四足机器人与人形 AI 机器人研发，产品面向电力巡检、应急救援、工厂巡检等复杂工业场景。公司强调重载、长续航和复杂地形适应能力，并在广东机器人产业链中持续推进产品化。</x:v>
       </x:c>
       <x:c r="M32" s="12" t="str">
-        <x:v>https://fysics.net/</x:v>
+        <x:v>https://www.gdlinxai.com/</x:v>
       </x:c>
       <x:c r="N32" s="12" t="str">
-        <x:v>电话：021-60197571；商务邮箱：fysics@fysics.ai；官网联系页：https://fysics.net/contact.html。</x:v>
+        <x:v>电话：17710125211；邮箱：info@linxai-tech.com；官网联系页：https://www.gdlinxai.com/h-col-109.html</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="12" t="str">
-        <x:v>蓝凌星通</x:v>
+        <x:v>安澜德健</x:v>
       </x:c>
       <x:c r="B33" s="12" t="str">
-        <x:v>卫星通信</x:v>
+        <x:v>医疗器械 / 心室辅助装置</x:v>
       </x:c>
       <x:c r="C33" s="13" t="n">
-        <x:v>46240.333333333336</x:v>
+        <x:v>46252.333333333336</x:v>
       </x:c>
       <x:c r="D33" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>近亿元人民币</x:v>
       </x:c>
       <x:c r="E33" s="12" t="str">
-        <x:v>股权融资</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F33" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G33" s="14"/>
       <x:c r="H33" s="12" t="str">
-        <x:v>启迪之星</x:v>
+        <x:v>启明创投</x:v>
       </x:c>
       <x:c r="I33" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E8%93%9D%E5%87%8C%E6%98%9F%E9%80%9A%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://www.qimingvc.com/cn/news/%E5%90%AF%E6%98%8E%E6%98%9F-%E5%AE%89%E6%BE%9C%E5%BE%B7%E5%81%A5%E5%AE%8C%E6%88%90%E8%BF%91%E4%BA%BF%E5%85%83a%E8%BD%AE%E8%9E%8D%E8%B5%84%EF%BC%8C%E5%90%AF%E6%98%8E%E5%88%9B%E6%8A%95%E7%8B%AC%E5%AE%B6%E6%8A%95%E8%B5%84</x:v>
       </x:c>
       <x:c r="J33" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46253.82167824074</x:v>
       </x:c>
       <x:c r="K33" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L33" s="12" t="str">
-        <x:v>蓝凌星通是蓝牙卫星系统服务商，利用低轨卫星为蓝牙终端提供低成本、低功耗的物联网连接和行业监测方案。其目标是把现有蓝牙终端延伸到传统地面网络覆盖不足的区域，服务户外、物流、资产追踪和行业监测等场景。</x:v>
+        <x:v>安澜德健（Enginprime Medical）专注经皮心室辅助装置（pVAD）研发，核心产品为 OpusOne™。公司围绕更小尺寸、更高流量的心室辅助系统推进中国注册临床试验与海外早期临床申报。</x:v>
       </x:c>
       <x:c r="M33" s="12" t="str">
-        <x:v>https://www.bluelinksatcom.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N33" s="12" t="str">
-        <x:v>电话：400-8818-251；商务邮箱：market@bluelinksatcom.com。</x:v>
+        <x:v>媒体邮箱：media@enginprime.com；投资者联系：info@voyagerscap.com</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="12" t="str">
-        <x:v>RoboParty（萝博派对）</x:v>
+        <x:v>亿兰科</x:v>
       </x:c>
       <x:c r="B34" s="12" t="str">
-        <x:v>具身智能 / 人形机器人</x:v>
+        <x:v>高端分析仪器 / 质谱仪</x:v>
       </x:c>
       <x:c r="C34" s="13" t="n">
-        <x:v>46238.333333333336</x:v>
+        <x:v>46245.333333333336</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
-        <x:v>近 5 亿元人民币</x:v>
+        <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E34" s="12" t="str">
-        <x:v>天使++轮及 Pre-A 轮</x:v>
+        <x:v>Pre-A 轮</x:v>
       </x:c>
       <x:c r="F34" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G34" s="14"/>
       <x:c r="H34" s="12" t="str">
-        <x:v>快科技（新浪财经转载）</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I34" s="16" t="str">
-        <x:v>https://finance.sina.com.cn/tech/roll/2026-08-04/doc-inimchzp5821502.shtml</x:v>
+        <x:v>https://news.pedaily.cn/202608/567473.shtml</x:v>
       </x:c>
       <x:c r="J34" s="15" t="n">
-        <x:v>46242.5</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K34" s="12" t="str">
-        <x:v>媒体交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L34" s="12" t="str">
-        <x:v>RoboParty 专注低成本、高性能双足人形机器人研发，并通过全栈开源建设机器人开发生态。公司公开机器人结构、电气、训练和部署等技术资料，希望降低研究者与开发者进入人形机器人研发的门槛，并推动软硬件协同迭代。</x:v>
+        <x:v>亿兰科专注工商业模块化光储系统和电力电子设备，围绕 PCS、混合逆变器、光储一体机与微电网管理系统开展研发和交付。公司产品服务工商业储能、分布式光伏和海外终端市场。</x:v>
       </x:c>
       <x:c r="M34" s="12" t="str">
-        <x:v>https://roboparty.com/</x:v>
+        <x:v>https://www.elecod.cn/</x:v>
       </x:c>
       <x:c r="N34" s="12" t="str">
-        <x:v>商务邮箱：contact@roboparty.com；开源技术交流 QQ 群：1078670917；官方 GitHub：https://github.com/Roboparty。</x:v>
+        <x:v>电话：0755-23050802；商务邮箱：marketing@elecod.com；人力邮箱：hr@elecod.com；官网联系页：https://www.elecod.cn/aboutus.html。</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="12" t="str">
-        <x:v>昉擎科技</x:v>
+        <x:v>诺因智能</x:v>
       </x:c>
       <x:c r="B35" s="12" t="str">
-        <x:v>AI 算力芯片</x:v>
+        <x:v>具身智能 / 消费级机器人</x:v>
       </x:c>
       <x:c r="C35" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>5 亿元人民币</x:v>
       </x:c>
       <x:c r="E35" s="12" t="str">
-        <x:v>A1 轮</x:v>
+        <x:v>天使++轮</x:v>
       </x:c>
       <x:c r="F35" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G35" s="14"/>
+      <x:c r="G35" s="14" t="n">
+        <x:v>50000</x:v>
+      </x:c>
       <x:c r="H35" s="12" t="str">
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I35" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%98%89%E6%93%8E%E7%A7%91%E6%8A%80%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202608/567457.shtml</x:v>
       </x:c>
       <x:c r="J35" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K35" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L35" s="12" t="str">
-        <x:v>昉擎科技是新一代智能计算系统企业，基于分离式架构和 4D Memory 理论，自主研发芯片、硬件系统与软件栈。公司重点解决 AI 计算系统的通用性、扩展性与工程化部署问题；本轮融资主要用于自研芯片和系统研发、规模化量产、软件生态建设及人才引进。</x:v>
+        <x:v>诺因智能聚焦家庭场景具身智能，围绕折叠双臂机器人及相关感知、执行和交互系统推进产品研发。公司目标是让机器人进入真实家庭环境，承担陪伴互动、整理和基础协作等任务。</x:v>
       </x:c>
       <x:c r="M35" s="12" t="str">
-        <x:v>未找到已核验官网</x:v>
+        <x:v>https://knowinai.com/</x:v>
       </x:c>
       <x:c r="N35" s="12" t="str">
-        <x:v>未找到公开商务联系方式</x:v>
+        <x:v>招聘邮箱：HR@knowin.ai；联系电话：17610340223；媒介合作：media@knowin.ai；官方联系页：https://knowinai.com/。</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="12" t="str">
-        <x:v>协鑫光电</x:v>
+        <x:v>星环聚能</x:v>
       </x:c>
       <x:c r="B36" s="12" t="str">
-        <x:v>钙钛矿光伏</x:v>
+        <x:v>可控聚变 / 清洁能源</x:v>
       </x:c>
       <x:c r="C36" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>超 1 亿元人民币</x:v>
+        <x:v>8.8 亿元人民币</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
-        <x:v>D1 轮</x:v>
+        <x:v>A++ 轮</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G36" s="14"/>
+      <x:c r="G36" s="14" t="n">
+        <x:v>88000</x:v>
+      </x:c>
       <x:c r="H36" s="12" t="str">
         <x:v>投资界</x:v>
       </x:c>
       <x:c r="I36" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%8D%8F%E9%91%AB%E5%85%89%E7%94%B5%20D1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202608/567446.shtml</x:v>
       </x:c>
       <x:c r="J36" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K36" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L36" s="12" t="str">
-        <x:v>协鑫光电主要从事大面积钙钛矿光伏组件的研发、生产及商业化应用。公司围绕钙钛矿材料、组件制备、封装可靠性和量产工艺推进技术迭代，面向下一代高效率光伏组件及其应用市场。</x:v>
+        <x:v>星环聚能专注可控核聚变相关技术和工程化系统，推动聚变能装备研发及商业化路径。公司面向清洁能源、长期稳定供能和能源转型场景，持续扩展实验和产业化能力。</x:v>
       </x:c>
       <x:c r="M36" s="12" t="str">
-        <x:v>https://www.gcl-perovskite.com/</x:v>
+        <x:v>https://startorus.cn/</x:v>
       </x:c>
       <x:c r="N36" s="12" t="str">
-        <x:v>官网公开电话：86-0512-57562287；官网联系页：https://www.gcl-power.com/contact.html。</x:v>
+        <x:v>电话：029-86041002；邮箱：business@startorus.cn；公司地址：上海市嘉定区澄浏公路52号39幢2楼JT109869室；官网联系页：https://startorus.cn/。</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
-        <x:v>主动科技</x:v>
+        <x:v>奇算光启</x:v>
       </x:c>
       <x:c r="B37" s="12" t="str">
-        <x:v>脑机接口</x:v>
+        <x:v>AI 光计算芯片</x:v>
       </x:c>
       <x:c r="C37" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
-        <x:v>3.3 亿元人民币</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E37" s="12" t="str">
-        <x:v>天使轮</x:v>
+        <x:v>天使轮及天使+轮</x:v>
       </x:c>
       <x:c r="F37" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G37" s="14" t="n">
-        <x:v>33000</x:v>
-      </x:c>
+      <x:c r="G37" s="14"/>
       <x:c r="H37" s="12" t="str">
-        <x:v>观点网</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I37" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E4%B8%BB%E5%8A%A8%E7%A7%91%E6%8A%80%203.3%E4%BA%BF%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202608/567453.shtml</x:v>
       </x:c>
       <x:c r="J37" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K37" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L37" s="12" t="str">
-        <x:v>主动科技是一家侵入式脑机接口技术研发与产业化企业，核心产品为“天枢”运动脑机接口。公开报道显示，公司成立于 2026 年 2 月，正推进高通道脑机系统、微纳加工平台与临床试验，目标是推动侵入式脑机接口从实验室验证走向医疗器械产业化。</x:v>
+        <x:v>奇算光启专注 AI 光计算芯片和光计算系统研发，试图用全光计算与集成光子技术突破传统电子芯片能效瓶颈。公司面向大模型和高性能计算底座，强调算力密度、功耗和系统扩展能力。</x:v>
       </x:c>
       <x:c r="M37" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1820,80 +1818,80 @@
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="12" t="str">
-        <x:v>西湖心辰</x:v>
+        <x:v>深度细胞</x:v>
       </x:c>
       <x:c r="B38" s="12" t="str">
-        <x:v>生成式 AI</x:v>
+        <x:v>AI 医疗 / 单细胞分析</x:v>
       </x:c>
       <x:c r="C38" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>近亿元人民币</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>B+ 轮</x:v>
+        <x:v>种子轮</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G38" s="14"/>
       <x:c r="H38" s="12" t="str">
-        <x:v>澎湃新闻</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I38" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E8%A5%BF%E6%B9%96%E5%BF%83%E8%BE%B0%20B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202608/567451.shtml</x:v>
       </x:c>
       <x:c r="J38" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K38" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L38" s="12" t="str">
-        <x:v>西湖心辰是一家生成式 AI 公司，研发西湖大模型及面向创作与企业场景的 AI 原生应用。公司将大模型能力用于内容生成、智能交互和行业工作流，强调模型能力与实际产品体验、企业落地场景的结合。</x:v>
+        <x:v>深度细胞聚焦 AI 制药与虚拟细胞建模，围绕单细胞分析、疾病机理和药物研发加速构建算法平台。公司目标是把细胞级计算能力用于新药发现和生物医学研究。</x:v>
       </x:c>
       <x:c r="M38" s="12" t="str">
-        <x:v>https://xinchenai.com/</x:v>
+        <x:v>未找到已核验官网</x:v>
       </x:c>
       <x:c r="N38" s="12" t="str">
-        <x:v>电话：400-8126-618；邮箱：support@xinchenai.com；地址：浙江省杭州市西湖区智强路428号云创镓谷6号楼6楼604室。</x:v>
+        <x:v>未找到公开商务联系方式</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="12" t="str">
-        <x:v>璨辰科技</x:v>
+        <x:v>橡木果机器人</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
-        <x:v>医疗 AI / 虚拟器官仿真</x:v>
+        <x:v>具身智能 / 人形机器人</x:v>
       </x:c>
       <x:c r="C39" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>数千万元人民币</x:v>
+        <x:v>未披露</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
-        <x:v>天使系列轮</x:v>
+        <x:v>天使轮</x:v>
       </x:c>
       <x:c r="F39" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G39" s="14"/>
       <x:c r="H39" s="12" t="str">
-        <x:v>雷峰网</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I39" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%92%A8%E8%BE%B0%E7%A7%91%E6%8A%80%20%E8%99%9A%E6%8B%9F%E5%99%A8%E5%AE%98%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202608/567448.shtml</x:v>
       </x:c>
       <x:c r="J39" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K39" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L39" s="12" t="str">
-        <x:v>璨辰科技聚焦系统级虚拟器官时空动态演化模型研发，构建从分子、细胞、组织到器官的全尺度 AI 数字孪生平台。其方案服务于新药临床前评价、发育毒性评估与疾病机制研究，并通过“仿真—湿实验—临床前验证”的数据闭环提升模型的产业转化价值。</x:v>
+        <x:v>橡木果机器人专注通用具身操作，围绕触觉感知、操作基座模型和机器人执行能力构建底层技术栈。公司强调自下而上的“本能驱动”路线，目标是让机器人在真实物理环境中稳定完成操作任务。</x:v>
       </x:c>
       <x:c r="M39" s="12" t="str">
         <x:v>未找到已核验官网</x:v>
@@ -1904,329 +1902,325 @@
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="12" t="str">
-        <x:v>鸿鹄航空</x:v>
+        <x:v>Noiz AI</x:v>
       </x:c>
       <x:c r="B40" s="12" t="str">
-        <x:v>航空航天</x:v>
+        <x:v>AI 语音 / 视听内容生成</x:v>
       </x:c>
       <x:c r="C40" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>7,000 万元人民币</x:v>
+        <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>种子轮</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G40" s="14" t="n">
-        <x:v>7000</x:v>
-      </x:c>
+      <x:c r="G40" s="14"/>
       <x:c r="H40" s="12" t="str">
-        <x:v>观点网</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I40" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E9%B8%BF%E9%B9%84%E8%88%AA%E7%A9%BA%207000%E4%B8%87%20A%E8%BD%AE&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.pedaily.cn/202608/567447.shtml</x:v>
       </x:c>
       <x:c r="J40" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K40" s="12" t="str">
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L40" s="12" t="str">
-        <x:v>青岛鸿鹄航空科技有限公司专注航空温控产品与服务，是海尔生物医疗控股子公司。公司围绕航空装备温度控制和相关系统服务开展产品研发，服务航空运行与专业运输等对环境控制要求较高的场景。</x:v>
+        <x:v>Noiz AI 提供文本转语音、声音克隆和语音设计能力，面向内容创作、配音、本地化和开发者 API 场景。其产品强调情感控制、低延迟生成和多语言语音输出，服务全球化音频工作流。</x:v>
       </x:c>
       <x:c r="M40" s="12" t="str">
-        <x:v>https://www.hbtempconaviation.com/</x:v>
+        <x:v>https://noiz.ai/</x:v>
       </x:c>
       <x:c r="N40" s="12" t="str">
-        <x:v>电话：+86-400-863-0863；邮箱：aviation@haierbiomedical.com；地址：青岛市高新区丰源路280号。</x:v>
+        <x:v>邮箱：contact@noiz.ai；官网联系页：https://noiz.ai/。</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="12" t="str">
-        <x:v>元育生物</x:v>
+        <x:v>飞声</x:v>
       </x:c>
       <x:c r="B41" s="12" t="str">
-        <x:v>生物医药</x:v>
+        <x:v>AI 助听器 / 医疗器械</x:v>
       </x:c>
       <x:c r="C41" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
-        <x:v>亿元人民币</x:v>
+        <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E41" s="12" t="str">
-        <x:v>A+ 轮</x:v>
+        <x:v>天使轮</x:v>
       </x:c>
       <x:c r="F41" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
-      <x:c r="G41" s="14" t="n">
-        <x:v>10000</x:v>
-      </x:c>
+      <x:c r="G41" s="14"/>
       <x:c r="H41" s="12" t="str">
-        <x:v>投资界</x:v>
+        <x:v>36氪</x:v>
       </x:c>
       <x:c r="I41" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%85%83%E8%82%B2%E7%94%9F%E7%89%A9%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E9%A3%9E%E5%A3%B0%20AI%20%E5%8A%A9%E5%90%AC%E5%99%A8%20%E5%A4%A9%E4%BD%BF%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J41" s="15" t="n">
-        <x:v>46241.479166666664</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K41" s="12" t="str">
-        <x:v>已核验</x:v>
+        <x:v>媒体与官网交叉核验</x:v>
       </x:c>
       <x:c r="L41" s="12" t="str">
-        <x:v>元育生物是微藻生物合成企业，开发可持续微藻基原料并提供定制化应用解决方案。公司以微藻培养、代谢调控和生物制造为技术基础，探索在食品营养、功能原料、日化与绿色消费品等领域的产业化应用。</x:v>
+        <x:v>飞声专注 AI 助听器与听力辅助产品，结合声学处理、语音增强和智能交互能力改善听障场景的佩戴体验。公司面向消费级与医疗级场景推进产品化，强调清晰拾音、降噪和更自然的听觉补偿。</x:v>
       </x:c>
       <x:c r="M41" s="12" t="str">
-        <x:v>https://www.protoga.com/</x:v>
+        <x:v>https://www.flysounds.cn/zh/</x:v>
       </x:c>
       <x:c r="N41" s="12" t="str">
-        <x:v>珠海：0756-8699334；北京：010-67866793；海外 BD：bd@protoga.com；国内销售：sales@protoga.com；地址：广东省珠海市香洲区南屏镇科技工业园屏北一路30号1栋2楼。</x:v>
+        <x:v>电话：15828225541；商务邮箱：jory@flysounds.com；地址：深圳市龙华区龙华街道清湖社区大和路356号金鼎盛科创园A栋18楼。</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="12" t="str">
-        <x:v>幺正量子</x:v>
+        <x:v>霍德生物</x:v>
       </x:c>
       <x:c r="B42" s="12" t="str">
-        <x:v>量子计算</x:v>
+        <x:v>细胞治疗 / 生物技术</x:v>
       </x:c>
       <x:c r="C42" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46244.333333333336</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
-        <x:v>数亿元人民币</x:v>
+        <x:v>近 2 亿元人民币</x:v>
       </x:c>
       <x:c r="E42" s="12" t="str">
-        <x:v>A 轮</x:v>
+        <x:v>C 轮首关</x:v>
       </x:c>
       <x:c r="F42" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G42" s="14"/>
       <x:c r="H42" s="12" t="str">
-        <x:v>大河财立方</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I42" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E5%B9%BA%E6%AD%A3%E9%87%8F%E5%AD%90%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E9%9C%8D%E5%BE%B7%E7%94%9F%E7%89%A9%20%E8%BF%91%202%20%E4%BA%BF%E5%85%83%20C%E8%BD%AE%20%E9%A6%96%E5%85%B3&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J42" s="15" t="n">
-        <x:v>46242.479166666664</x:v>
+        <x:v>46245.44097222222</x:v>
       </x:c>
       <x:c r="K42" s="12" t="str">
-        <x:v>待官网交叉核验</x:v>
+        <x:v>媒体与公开工商信息交叉核验</x:v>
       </x:c>
       <x:c r="L42" s="12" t="str">
-        <x:v>幺正量子是一家离子阱量子计算企业，提供量子计算系统、设备器件、云服务和行业解决方案。公司围绕离子阱硬件、量子控制、算法与行业应用推进全栈研发，服务科研、教育和量子计算产业化需求。</x:v>
+        <x:v>霍德生物工程有限公司聚焦细胞治疗和再生医学相关技术与产品，围绕研发、工艺和临床转化推进管线建设。公司在公开页面中长期披露研发动态与产品进展，面向生物医药产业化需求。</x:v>
       </x:c>
       <x:c r="M42" s="12" t="str">
-        <x:v>https://www.unitqc.com/</x:v>
+        <x:v>https://www.hopstem.com/</x:v>
       </x:c>
       <x:c r="N42" s="12" t="str">
-        <x:v>商务邮箱：business@unitqc.com；电话：15391985489；地址：安徽省合肥市高新区望江西路900号中安创谷科技园一期B1栋1-2层。</x:v>
+        <x:v>电话：0571-88197776；邮箱：info@hopstem.com；官网联系页：https://www.hopstem.com/。</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="12" t="str">
-        <x:v>恺望数据</x:v>
+        <x:v>可灵 AI</x:v>
       </x:c>
       <x:c r="B43" s="12" t="str">
-        <x:v>AI 数据服务</x:v>
+        <x:v>AI 视频大模型</x:v>
       </x:c>
       <x:c r="C43" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46241.333333333336</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
-        <x:v>逾亿元人民币</x:v>
+        <x:v>近 30 亿美元</x:v>
       </x:c>
       <x:c r="E43" s="12" t="str">
         <x:v>未披露</x:v>
       </x:c>
       <x:c r="F43" s="12" t="str">
-        <x:v>CNY</x:v>
+        <x:v>USD</x:v>
       </x:c>
       <x:c r="G43" s="14"/>
       <x:c r="H43" s="12" t="str">
-        <x:v>封面新闻</x:v>
+        <x:v>新华网 / 经济参考报</x:v>
       </x:c>
       <x:c r="I43" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%81%BA%E6%9C%9B%E6%95%B0%E6%8D%AE%20%E9%80%BE%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://www.news.cn/tech/20260807/1605ef446e5045b7ba0ee55245ce731c/c.html</x:v>
       </x:c>
       <x:c r="J43" s="15" t="n">
-        <x:v>46242.479166666664</x:v>
+        <x:v>46242.48541666667</x:v>
       </x:c>
       <x:c r="K43" s="12" t="str">
-        <x:v>待官网交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L43" s="12" t="str">
-        <x:v>恺望数据为车企、自动驾驶及 AI 企业提供一站式数据解决方案和自动化数据生产能力。其服务覆盖数据采集、清洗、标注、质检和管理，重点支持自动驾驶、具身智能与大模型训练中的规模化高质量数据供给。</x:v>
+        <x:v>可灵 AI 是面向视频生成与创作的 AI 大模型产品，支持文本、图片等输入驱动的视频内容生成和编辑。产品服务广告创意、影视内容、社交媒体和商业化营销等场景，重点提升视频生成的一致性、可控性和创作效率。</x:v>
       </x:c>
       <x:c r="M43" s="12" t="str">
-        <x:v>https://admin.d.konvery.com/</x:v>
+        <x:v>https://klingai.com/</x:v>
       </x:c>
       <x:c r="N43" s="12" t="str">
-        <x:v>官方产品平台：https://admin.d.konvery.com/；官网未公开完整商务电话或邮箱，可通过平台申请试用或联系。</x:v>
+        <x:v>商务联系：官网联系页</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="12" t="str">
-        <x:v>求是光谱</x:v>
+        <x:v>矩阵起源</x:v>
       </x:c>
       <x:c r="B44" s="12" t="str">
-        <x:v>光谱检测</x:v>
+        <x:v>企业级 AI 基础设施</x:v>
       </x:c>
       <x:c r="C44" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46240.333333333336</x:v>
       </x:c>
       <x:c r="D44" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>超 1,000 万美元</x:v>
       </x:c>
       <x:c r="E44" s="12" t="str">
-        <x:v>B++ 轮</x:v>
+        <x:v>A 轮</x:v>
       </x:c>
       <x:c r="F44" s="12" t="str">
-        <x:v>CNY</x:v>
-      </x:c>
-      <x:c r="G44" s="14"/>
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G44" s="14" t="n">
+        <x:v>7200</x:v>
+      </x:c>
       <x:c r="H44" s="12" t="str">
-        <x:v>新浪财经</x:v>
+        <x:v>投资界</x:v>
       </x:c>
       <x:c r="I44" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%B1%82%E6%98%AF%E5%85%89%E8%B0%B1%20B%2B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E7%9F%A9%E9%98%B5%E8%B5%B7%E6%BA%90%20%E8%B6%85%E5%8D%83%E4%B8%87%E7%BE%8E%E5%85%83%20A%E8%BD%AE%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J44" s="15" t="n">
-        <x:v>46242.479166666664</x:v>
+        <x:v>46241.479166666664</x:v>
       </x:c>
       <x:c r="K44" s="12" t="str">
-        <x:v>待官网交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L44" s="12" t="str">
-        <x:v>求是光谱从事多光谱成像芯片、光谱应用方案及光谱大数据研发，为智能终端、汽车电子、医疗和环境监测等场景提供产品与服务。公司将光谱感知能力嵌入硬件和软件方案，用于物质识别、成分分析和复杂环境下的智能检测。</x:v>
+        <x:v>矩阵起源专注 AI 原生数据基础设施，提供多模态数据处理、数据库与企业级 AI 数据底座产品及解决方案。其产品面向企业在结构化、非结构化和向量数据之间建立统一的数据管理与计算能力，为模型训练、知识检索和 AI 应用部署提供底层支撑。</x:v>
       </x:c>
       <x:c r="M44" s="12" t="str">
-        <x:v>https://www.qsspec.com/</x:v>
+        <x:v>https://matrixorigin.cn/</x:v>
       </x:c>
       <x:c r="N44" s="12" t="str">
-        <x:v>电话：0431-88882290；商务联系人：冯硕，18343025432，fengshuo@qsspec.com；展会公开邮箱：hanying@qsspec.com。</x:v>
+        <x:v>商务邮箱：contact@matrixorigin.cn。</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="12" t="str">
-        <x:v>熵简科技</x:v>
+        <x:v>为光能源</x:v>
       </x:c>
       <x:c r="B45" s="12" t="str">
-        <x:v>企业软件 / 数据智能</x:v>
+        <x:v>电力电子 / 固态变压器</x:v>
       </x:c>
       <x:c r="C45" s="13" t="n">
-        <x:v>46237.333333333336</x:v>
+        <x:v>46240.333333333336</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
-        <x:v>C 轮</x:v>
+        <x:v>B 轮</x:v>
       </x:c>
       <x:c r="F45" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G45" s="14"/>
       <x:c r="H45" s="12" t="str">
-        <x:v>新浪财经</x:v>
+        <x:v>中国网</x:v>
       </x:c>
       <x:c r="I45" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%86%B5%E7%AE%80%E7%A7%91%E6%8A%80%20C%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E4%B8%BA%E5%85%89%E8%83%BD%E6%BA%90%20B%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J45" s="15" t="n">
-        <x:v>46242.479166666664</x:v>
+        <x:v>46241.479166666664</x:v>
       </x:c>
       <x:c r="K45" s="12" t="str">
-        <x:v>待官网交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L45" s="12" t="str">
-        <x:v>熵简科技是面向金融资管行业的数字基础设施与数据智能服务商，提供另类数据、知识图谱和全域数据中台等能力。公司自主研发大数据分析引擎，帮助金融机构处理多源异构数据、构建标准化 API，并支持投研、风险管理和业务决策工作流。</x:v>
+        <x:v>西安为光能源科技有限公司聚焦固态变压器（SST）等新型电力电子装备及能源互联网解决方案。公司瞄准算力中心、电动交通、新型配网和储能等高功率密度场景，通过电能变换、控制和系统集成提升供配电效率与灵活性。</x:v>
       </x:c>
       <x:c r="M45" s="12" t="str">
-        <x:v>https://www.valuesimplex.com/</x:v>
+        <x:v>https://www.weiguangenergy.com/</x:v>
       </x:c>
       <x:c r="N45" s="12" t="str">
-        <x:v>官网提供业务咨询入口；暂未检索到可交叉确认的公开商务电话或邮箱。</x:v>
+        <x:v>服务热线：400-868-6988；商务邮箱（官网公开）：wangjuan0509@foxmail.com；地址：陕西省西安市高新区毕原二路3号先导院南区5-6号楼；公众号：WGenergy；在线留言：官网联系页。</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="12" t="str">
-        <x:v>灏存科技</x:v>
+        <x:v>飞捷科思</x:v>
       </x:c>
       <x:c r="B46" s="12" t="str">
-        <x:v>硬科技</x:v>
+        <x:v>半导体</x:v>
       </x:c>
       <x:c r="C46" s="13" t="n">
-        <x:v>46235.333333333336</x:v>
+        <x:v>46240.333333333336</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
-        <x:v>未披露</x:v>
+        <x:v>数亿元人民币</x:v>
       </x:c>
       <x:c r="E46" s="12" t="str">
-        <x:v>A+ 轮</x:v>
+        <x:v>A1 轮</x:v>
       </x:c>
       <x:c r="F46" s="12" t="str">
         <x:v>CNY</x:v>
       </x:c>
       <x:c r="G46" s="14"/>
       <x:c r="H46" s="12" t="str">
-        <x:v>新浪财经</x:v>
+        <x:v>观点网</x:v>
       </x:c>
       <x:c r="I46" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E7%81%8F%E5%AD%98%E7%A7%91%E6%8A%80%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E9%A3%9E%E6%8D%B7%E7%A7%91%E6%80%9D%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J46" s="15" t="n">
-        <x:v>46242.479166666664</x:v>
+        <x:v>46241.479166666664</x:v>
       </x:c>
       <x:c r="K46" s="12" t="str">
-        <x:v>待官网交叉核验</x:v>
+        <x:v>已核验</x:v>
       </x:c>
       <x:c r="L46" s="12" t="str">
-        <x:v>灏存科技从事人工智能穿戴型肢体动作识别软硬件技术研发，应用于 VR/AR/MR、电影工业和人形机器人运动感知场景。公司以穿戴式传感、人体动作捕捉和算法识别为核心，使虚拟交互、数字内容生产和机器人训练获得更细粒度的运动数据。</x:v>
+        <x:v>飞捷科思以高精度实时物理仿真引擎为核心，研发面向具身智能和人形机器人的物理智能技术与产品。其能力重点在于让机器人在虚拟环境中完成动力学、接触和运动策略验证，以缩短从算法训练到真实机器部署的迭代周期。</x:v>
       </x:c>
       <x:c r="M46" s="12" t="str">
-        <x:v>https://www.hexacercle.com/</x:v>
+        <x:v>https://fysics.net/</x:v>
       </x:c>
       <x:c r="N46" s="12" t="str">
-        <x:v>商务合作：+86 13349933396；邮箱：mike@hexacercle.com；武汉总部：武汉东湖高新区关东街道华工园三路湖北青创园4栋801。</x:v>
+        <x:v>电话：021-60197571；商务邮箱：fysics@fysics.ai；官网联系页：https://fysics.net/contact.html。</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="12" t="str">
-        <x:v>月之暗面（Kimi）</x:v>
+        <x:v>蓝凌星通</x:v>
       </x:c>
       <x:c r="B47" s="12" t="str">
-        <x:v>大模型</x:v>
+        <x:v>卫星通信</x:v>
       </x:c>
       <x:c r="C47" s="13" t="n">
-        <x:v>46234.333333333336</x:v>
+        <x:v>46240.333333333336</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
-        <x:v>超 35 亿美元</x:v>
+        <x:v>数千万元人民币</x:v>
       </x:c>
       <x:c r="E47" s="12" t="str">
-        <x:v>F 轮</x:v>
+        <x:v>股权融资</x:v>
       </x:c>
       <x:c r="F47" s="12" t="str">
-        <x:v>USD</x:v>
-      </x:c>
-      <x:c r="G47" s="14" t="n">
-        <x:v>2520000</x:v>
-      </x:c>
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G47" s="14"/>
       <x:c r="H47" s="12" t="str">
-        <x:v>创业邦</x:v>
+        <x:v>启迪之星</x:v>
       </x:c>
       <x:c r="I47" s="16" t="str">
-        <x:v>https://news.google.com/search?q=%E6%9C%88%E4%B9%8B%E6%9A%97%E9%9D%A2%20F%E8%BD%AE%2035%E4%BA%BF%E7%BE%8E%E5%85%83&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+        <x:v>https://news.google.com/search?q=%E8%93%9D%E5%87%8C%E6%98%9F%E9%80%9A%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
       </x:c>
       <x:c r="J47" s="15" t="n">
         <x:v>46241.479166666664</x:v>
@@ -2235,12 +2229,608 @@
         <x:v>已核验</x:v>
       </x:c>
       <x:c r="L47" s="12" t="str">
+        <x:v>蓝凌星通是蓝牙卫星系统服务商，利用低轨卫星为蓝牙终端提供低成本、低功耗的物联网连接和行业监测方案。其目标是把现有蓝牙终端延伸到传统地面网络覆盖不足的区域，服务户外、物流、资产追踪和行业监测等场景。</x:v>
+      </x:c>
+      <x:c r="M47" s="12" t="str">
+        <x:v>https://www.bluelinksatcom.com/</x:v>
+      </x:c>
+      <x:c r="N47" s="12" t="str">
+        <x:v>电话：400-8818-251；商务邮箱：market@bluelinksatcom.com。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
+      <x:c r="A48" s="12" t="str">
+        <x:v>RoboParty（萝博派对）</x:v>
+      </x:c>
+      <x:c r="B48" s="12" t="str">
+        <x:v>具身智能 / 人形机器人</x:v>
+      </x:c>
+      <x:c r="C48" s="13" t="n">
+        <x:v>46238.333333333336</x:v>
+      </x:c>
+      <x:c r="D48" s="12" t="str">
+        <x:v>近 5 亿元人民币</x:v>
+      </x:c>
+      <x:c r="E48" s="12" t="str">
+        <x:v>天使++轮及 Pre-A 轮</x:v>
+      </x:c>
+      <x:c r="F48" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G48" s="14"/>
+      <x:c r="H48" s="12" t="str">
+        <x:v>快科技（新浪财经转载）</x:v>
+      </x:c>
+      <x:c r="I48" s="16" t="str">
+        <x:v>https://finance.sina.com.cn/tech/roll/2026-08-04/doc-inimchzp5821502.shtml</x:v>
+      </x:c>
+      <x:c r="J48" s="15" t="n">
+        <x:v>46242.5</x:v>
+      </x:c>
+      <x:c r="K48" s="12" t="str">
+        <x:v>媒体交叉核验</x:v>
+      </x:c>
+      <x:c r="L48" s="12" t="str">
+        <x:v>RoboParty 专注低成本、高性能双足人形机器人研发，并通过全栈开源建设机器人开发生态。公司公开机器人结构、电气、训练和部署等技术资料，希望降低研究者与开发者进入人形机器人研发的门槛，并推动软硬件协同迭代。</x:v>
+      </x:c>
+      <x:c r="M48" s="12" t="str">
+        <x:v>https://roboparty.com/</x:v>
+      </x:c>
+      <x:c r="N48" s="12" t="str">
+        <x:v>商务邮箱：contact@roboparty.com；开源技术交流 QQ 群：1078670917；官方 GitHub：https://github.com/Roboparty。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
+      <x:c r="A49" s="12" t="str">
+        <x:v>昉擎科技</x:v>
+      </x:c>
+      <x:c r="B49" s="12" t="str">
+        <x:v>AI 算力芯片</x:v>
+      </x:c>
+      <x:c r="C49" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D49" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="E49" s="12" t="str">
+        <x:v>A1 轮</x:v>
+      </x:c>
+      <x:c r="F49" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G49" s="14"/>
+      <x:c r="H49" s="12" t="str">
+        <x:v>投资界</x:v>
+      </x:c>
+      <x:c r="I49" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E6%98%89%E6%93%8E%E7%A7%91%E6%8A%80%20A1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J49" s="15" t="n">
+        <x:v>46241.479166666664</x:v>
+      </x:c>
+      <x:c r="K49" s="12" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="L49" s="12" t="str">
+        <x:v>昉擎科技是新一代智能计算系统企业，基于分离式架构和 4D Memory 理论，自主研发芯片、硬件系统与软件栈。公司重点解决 AI 计算系统的通用性、扩展性与工程化部署问题；本轮融资主要用于自研芯片和系统研发、规模化量产、软件生态建设及人才引进。</x:v>
+      </x:c>
+      <x:c r="M49" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N49" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
+      <x:c r="A50" s="12" t="str">
+        <x:v>协鑫光电</x:v>
+      </x:c>
+      <x:c r="B50" s="12" t="str">
+        <x:v>钙钛矿光伏</x:v>
+      </x:c>
+      <x:c r="C50" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D50" s="12" t="str">
+        <x:v>超 1 亿元人民币</x:v>
+      </x:c>
+      <x:c r="E50" s="12" t="str">
+        <x:v>D1 轮</x:v>
+      </x:c>
+      <x:c r="F50" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G50" s="14"/>
+      <x:c r="H50" s="12" t="str">
+        <x:v>投资界</x:v>
+      </x:c>
+      <x:c r="I50" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E5%8D%8F%E9%91%AB%E5%85%89%E7%94%B5%20D1%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J50" s="15" t="n">
+        <x:v>46241.479166666664</x:v>
+      </x:c>
+      <x:c r="K50" s="12" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="L50" s="12" t="str">
+        <x:v>协鑫光电主要从事大面积钙钛矿光伏组件的研发、生产及商业化应用。公司围绕钙钛矿材料、组件制备、封装可靠性和量产工艺推进技术迭代，面向下一代高效率光伏组件及其应用市场。</x:v>
+      </x:c>
+      <x:c r="M50" s="12" t="str">
+        <x:v>https://www.gcl-perovskite.com/</x:v>
+      </x:c>
+      <x:c r="N50" s="12" t="str">
+        <x:v>官网公开电话：86-0512-57562287；官网联系页：https://www.gcl-power.com/contact.html。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
+      <x:c r="A51" s="12" t="str">
+        <x:v>主动科技</x:v>
+      </x:c>
+      <x:c r="B51" s="12" t="str">
+        <x:v>脑机接口</x:v>
+      </x:c>
+      <x:c r="C51" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D51" s="12" t="str">
+        <x:v>3.3 亿元人民币</x:v>
+      </x:c>
+      <x:c r="E51" s="12" t="str">
+        <x:v>天使轮</x:v>
+      </x:c>
+      <x:c r="F51" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G51" s="14" t="n">
+        <x:v>33000</x:v>
+      </x:c>
+      <x:c r="H51" s="12" t="str">
+        <x:v>观点网</x:v>
+      </x:c>
+      <x:c r="I51" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E4%B8%BB%E5%8A%A8%E7%A7%91%E6%8A%80%203.3%E4%BA%BF%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J51" s="15" t="n">
+        <x:v>46241.479166666664</x:v>
+      </x:c>
+      <x:c r="K51" s="12" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="L51" s="12" t="str">
+        <x:v>主动科技是一家侵入式脑机接口技术研发与产业化企业，核心产品为“天枢”运动脑机接口。公开报道显示，公司成立于 2026 年 2 月，正推进高通道脑机系统、微纳加工平台与临床试验，目标是推动侵入式脑机接口从实验室验证走向医疗器械产业化。</x:v>
+      </x:c>
+      <x:c r="M51" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N51" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="A52" s="12" t="str">
+        <x:v>西湖心辰</x:v>
+      </x:c>
+      <x:c r="B52" s="12" t="str">
+        <x:v>生成式 AI</x:v>
+      </x:c>
+      <x:c r="C52" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D52" s="12" t="str">
+        <x:v>数亿元人民币</x:v>
+      </x:c>
+      <x:c r="E52" s="12" t="str">
+        <x:v>B+ 轮</x:v>
+      </x:c>
+      <x:c r="F52" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G52" s="14"/>
+      <x:c r="H52" s="12" t="str">
+        <x:v>澎湃新闻</x:v>
+      </x:c>
+      <x:c r="I52" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E8%A5%BF%E6%B9%96%E5%BF%83%E8%BE%B0%20B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J52" s="15" t="n">
+        <x:v>46241.479166666664</x:v>
+      </x:c>
+      <x:c r="K52" s="12" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="L52" s="12" t="str">
+        <x:v>西湖心辰是一家生成式 AI 公司，研发西湖大模型及面向创作与企业场景的 AI 原生应用。公司将大模型能力用于内容生成、智能交互和行业工作流，强调模型能力与实际产品体验、企业落地场景的结合。</x:v>
+      </x:c>
+      <x:c r="M52" s="12" t="str">
+        <x:v>https://xinchenai.com/</x:v>
+      </x:c>
+      <x:c r="N52" s="12" t="str">
+        <x:v>电话：400-8126-618；邮箱：support@xinchenai.com；地址：浙江省杭州市西湖区智强路428号云创镓谷6号楼6楼604室。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="12" t="str">
+        <x:v>璨辰科技</x:v>
+      </x:c>
+      <x:c r="B53" s="12" t="str">
+        <x:v>医疗 AI / 虚拟器官仿真</x:v>
+      </x:c>
+      <x:c r="C53" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D53" s="12" t="str">
+        <x:v>数千万元人民币</x:v>
+      </x:c>
+      <x:c r="E53" s="12" t="str">
+        <x:v>天使系列轮</x:v>
+      </x:c>
+      <x:c r="F53" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G53" s="14"/>
+      <x:c r="H53" s="12" t="str">
+        <x:v>雷峰网</x:v>
+      </x:c>
+      <x:c r="I53" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E7%92%A8%E8%BE%B0%E7%A7%91%E6%8A%80%20%E8%99%9A%E6%8B%9F%E5%99%A8%E5%AE%98%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J53" s="15" t="n">
+        <x:v>46241.479166666664</x:v>
+      </x:c>
+      <x:c r="K53" s="12" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="L53" s="12" t="str">
+        <x:v>璨辰科技聚焦系统级虚拟器官时空动态演化模型研发，构建从分子、细胞、组织到器官的全尺度 AI 数字孪生平台。其方案服务于新药临床前评价、发育毒性评估与疾病机制研究，并通过“仿真—湿实验—临床前验证”的数据闭环提升模型的产业转化价值。</x:v>
+      </x:c>
+      <x:c r="M53" s="12" t="str">
+        <x:v>未找到已核验官网</x:v>
+      </x:c>
+      <x:c r="N53" s="12" t="str">
+        <x:v>未找到公开商务联系方式</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="A54" s="12" t="str">
+        <x:v>鸿鹄航空</x:v>
+      </x:c>
+      <x:c r="B54" s="12" t="str">
+        <x:v>航空航天</x:v>
+      </x:c>
+      <x:c r="C54" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D54" s="12" t="str">
+        <x:v>7,000 万元人民币</x:v>
+      </x:c>
+      <x:c r="E54" s="12" t="str">
+        <x:v>A 轮</x:v>
+      </x:c>
+      <x:c r="F54" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G54" s="14" t="n">
+        <x:v>7000</x:v>
+      </x:c>
+      <x:c r="H54" s="12" t="str">
+        <x:v>观点网</x:v>
+      </x:c>
+      <x:c r="I54" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E9%B8%BF%E9%B9%84%E8%88%AA%E7%A9%BA%207000%E4%B8%87%20A%E8%BD%AE&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J54" s="15" t="n">
+        <x:v>46241.479166666664</x:v>
+      </x:c>
+      <x:c r="K54" s="12" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="L54" s="12" t="str">
+        <x:v>青岛鸿鹄航空科技有限公司专注航空温控产品与服务，是海尔生物医疗控股子公司。公司围绕航空装备温度控制和相关系统服务开展产品研发，服务航空运行与专业运输等对环境控制要求较高的场景。</x:v>
+      </x:c>
+      <x:c r="M54" s="12" t="str">
+        <x:v>https://www.hbtempconaviation.com/</x:v>
+      </x:c>
+      <x:c r="N54" s="12" t="str">
+        <x:v>电话：+86-400-863-0863；邮箱：aviation@haierbiomedical.com；地址：青岛市高新区丰源路280号。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
+      <x:c r="A55" s="12" t="str">
+        <x:v>元育生物</x:v>
+      </x:c>
+      <x:c r="B55" s="12" t="str">
+        <x:v>生物医药</x:v>
+      </x:c>
+      <x:c r="C55" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D55" s="12" t="str">
+        <x:v>亿元人民币</x:v>
+      </x:c>
+      <x:c r="E55" s="12" t="str">
+        <x:v>A+ 轮</x:v>
+      </x:c>
+      <x:c r="F55" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G55" s="14" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="H55" s="12" t="str">
+        <x:v>投资界</x:v>
+      </x:c>
+      <x:c r="I55" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E5%85%83%E8%82%B2%E7%94%9F%E7%89%A9%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J55" s="15" t="n">
+        <x:v>46241.479166666664</x:v>
+      </x:c>
+      <x:c r="K55" s="12" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="L55" s="12" t="str">
+        <x:v>元育生物是微藻生物合成企业，开发可持续微藻基原料并提供定制化应用解决方案。公司以微藻培养、代谢调控和生物制造为技术基础，探索在食品营养、功能原料、日化与绿色消费品等领域的产业化应用。</x:v>
+      </x:c>
+      <x:c r="M55" s="12" t="str">
+        <x:v>https://www.protoga.com/</x:v>
+      </x:c>
+      <x:c r="N55" s="12" t="str">
+        <x:v>珠海：0756-8699334；北京：010-67866793；海外 BD：bd@protoga.com；国内销售：sales@protoga.com；地址：广东省珠海市香洲区南屏镇科技工业园屏北一路30号1栋2楼。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
+      <x:c r="A56" s="12" t="str">
+        <x:v>幺正量子</x:v>
+      </x:c>
+      <x:c r="B56" s="12" t="str">
+        <x:v>量子计算</x:v>
+      </x:c>
+      <x:c r="C56" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D56" s="12" t="str">
+        <x:v>数亿元人民币</x:v>
+      </x:c>
+      <x:c r="E56" s="12" t="str">
+        <x:v>A 轮</x:v>
+      </x:c>
+      <x:c r="F56" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G56" s="14"/>
+      <x:c r="H56" s="12" t="str">
+        <x:v>大河财立方</x:v>
+      </x:c>
+      <x:c r="I56" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E5%B9%BA%E6%AD%A3%E9%87%8F%E5%AD%90%20A%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J56" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K56" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L56" s="12" t="str">
+        <x:v>幺正量子是一家离子阱量子计算企业，提供量子计算系统、设备器件、云服务和行业解决方案。公司围绕离子阱硬件、量子控制、算法与行业应用推进全栈研发，服务科研、教育和量子计算产业化需求。</x:v>
+      </x:c>
+      <x:c r="M56" s="12" t="str">
+        <x:v>https://www.unitqc.com/</x:v>
+      </x:c>
+      <x:c r="N56" s="12" t="str">
+        <x:v>商务邮箱：business@unitqc.com；电话：15391985489；地址：安徽省合肥市高新区望江西路900号中安创谷科技园一期B1栋1-2层。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
+      <x:c r="A57" s="12" t="str">
+        <x:v>恺望数据</x:v>
+      </x:c>
+      <x:c r="B57" s="12" t="str">
+        <x:v>AI 数据服务</x:v>
+      </x:c>
+      <x:c r="C57" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D57" s="12" t="str">
+        <x:v>逾亿元人民币</x:v>
+      </x:c>
+      <x:c r="E57" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="F57" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G57" s="14"/>
+      <x:c r="H57" s="12" t="str">
+        <x:v>封面新闻</x:v>
+      </x:c>
+      <x:c r="I57" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E6%81%BA%E6%9C%9B%E6%95%B0%E6%8D%AE%20%E9%80%BE%E4%BA%BF%E5%85%83%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J57" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K57" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L57" s="12" t="str">
+        <x:v>恺望数据为车企、自动驾驶及 AI 企业提供一站式数据解决方案和自动化数据生产能力。其服务覆盖数据采集、清洗、标注、质检和管理，重点支持自动驾驶、具身智能与大模型训练中的规模化高质量数据供给。</x:v>
+      </x:c>
+      <x:c r="M57" s="12" t="str">
+        <x:v>https://admin.d.konvery.com/</x:v>
+      </x:c>
+      <x:c r="N57" s="12" t="str">
+        <x:v>官方产品平台：https://admin.d.konvery.com/；官网未公开完整商务电话或邮箱，可通过平台申请试用或联系。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="15" hidden="0" customHeight="1">
+      <x:c r="A58" s="12" t="str">
+        <x:v>求是光谱</x:v>
+      </x:c>
+      <x:c r="B58" s="12" t="str">
+        <x:v>光谱检测</x:v>
+      </x:c>
+      <x:c r="C58" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D58" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="E58" s="12" t="str">
+        <x:v>B++ 轮</x:v>
+      </x:c>
+      <x:c r="F58" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G58" s="14"/>
+      <x:c r="H58" s="12" t="str">
+        <x:v>新浪财经</x:v>
+      </x:c>
+      <x:c r="I58" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E6%B1%82%E6%98%AF%E5%85%89%E8%B0%B1%20B%2B%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J58" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K58" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L58" s="12" t="str">
+        <x:v>求是光谱从事多光谱成像芯片、光谱应用方案及光谱大数据研发，为智能终端、汽车电子、医疗和环境监测等场景提供产品与服务。公司将光谱感知能力嵌入硬件和软件方案，用于物质识别、成分分析和复杂环境下的智能检测。</x:v>
+      </x:c>
+      <x:c r="M58" s="12" t="str">
+        <x:v>https://www.qsspec.com/</x:v>
+      </x:c>
+      <x:c r="N58" s="12" t="str">
+        <x:v>电话：0431-88882290；商务联系人：冯硕，18343025432，fengshuo@qsspec.com；展会公开邮箱：hanying@qsspec.com。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="15" hidden="0" customHeight="1">
+      <x:c r="A59" s="12" t="str">
+        <x:v>熵简科技</x:v>
+      </x:c>
+      <x:c r="B59" s="12" t="str">
+        <x:v>企业软件 / 数据智能</x:v>
+      </x:c>
+      <x:c r="C59" s="13" t="n">
+        <x:v>46237.333333333336</x:v>
+      </x:c>
+      <x:c r="D59" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="E59" s="12" t="str">
+        <x:v>C 轮</x:v>
+      </x:c>
+      <x:c r="F59" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G59" s="14"/>
+      <x:c r="H59" s="12" t="str">
+        <x:v>新浪财经</x:v>
+      </x:c>
+      <x:c r="I59" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E7%86%B5%E7%AE%80%E7%A7%91%E6%8A%80%20C%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J59" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K59" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L59" s="12" t="str">
+        <x:v>熵简科技是面向金融资管行业的数字基础设施与数据智能服务商，提供另类数据、知识图谱和全域数据中台等能力。公司自主研发大数据分析引擎，帮助金融机构处理多源异构数据、构建标准化 API，并支持投研、风险管理和业务决策工作流。</x:v>
+      </x:c>
+      <x:c r="M59" s="12" t="str">
+        <x:v>https://www.valuesimplex.com/</x:v>
+      </x:c>
+      <x:c r="N59" s="12" t="str">
+        <x:v>官网提供业务咨询入口；暂未检索到可交叉确认的公开商务电话或邮箱。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="15" hidden="0" customHeight="1">
+      <x:c r="A60" s="12" t="str">
+        <x:v>灏存科技</x:v>
+      </x:c>
+      <x:c r="B60" s="12" t="str">
+        <x:v>硬科技</x:v>
+      </x:c>
+      <x:c r="C60" s="13" t="n">
+        <x:v>46235.333333333336</x:v>
+      </x:c>
+      <x:c r="D60" s="12" t="str">
+        <x:v>未披露</x:v>
+      </x:c>
+      <x:c r="E60" s="12" t="str">
+        <x:v>A+ 轮</x:v>
+      </x:c>
+      <x:c r="F60" s="12" t="str">
+        <x:v>CNY</x:v>
+      </x:c>
+      <x:c r="G60" s="14"/>
+      <x:c r="H60" s="12" t="str">
+        <x:v>新浪财经</x:v>
+      </x:c>
+      <x:c r="I60" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E7%81%8F%E5%AD%98%E7%A7%91%E6%8A%80%20A%2B%20%E8%BD%AE%20%E8%9E%8D%E8%B5%84&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J60" s="15" t="n">
+        <x:v>46242.479166666664</x:v>
+      </x:c>
+      <x:c r="K60" s="12" t="str">
+        <x:v>待官网交叉核验</x:v>
+      </x:c>
+      <x:c r="L60" s="12" t="str">
+        <x:v>灏存科技从事人工智能穿戴型肢体动作识别软硬件技术研发，应用于 VR/AR/MR、电影工业和人形机器人运动感知场景。公司以穿戴式传感、人体动作捕捉和算法识别为核心，使虚拟交互、数字内容生产和机器人训练获得更细粒度的运动数据。</x:v>
+      </x:c>
+      <x:c r="M60" s="12" t="str">
+        <x:v>https://www.hexacercle.com/</x:v>
+      </x:c>
+      <x:c r="N60" s="12" t="str">
+        <x:v>商务合作：+86 13349933396；邮箱：mike@hexacercle.com；武汉总部：武汉东湖高新区关东街道华工园三路湖北青创园4栋801。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="15" hidden="0" customHeight="1">
+      <x:c r="A61" s="12" t="str">
+        <x:v>月之暗面（Kimi）</x:v>
+      </x:c>
+      <x:c r="B61" s="12" t="str">
+        <x:v>大模型</x:v>
+      </x:c>
+      <x:c r="C61" s="13" t="n">
+        <x:v>46234.333333333336</x:v>
+      </x:c>
+      <x:c r="D61" s="12" t="str">
+        <x:v>超 35 亿美元</x:v>
+      </x:c>
+      <x:c r="E61" s="12" t="str">
+        <x:v>F 轮</x:v>
+      </x:c>
+      <x:c r="F61" s="12" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="G61" s="14" t="n">
+        <x:v>2520000</x:v>
+      </x:c>
+      <x:c r="H61" s="12" t="str">
+        <x:v>创业邦</x:v>
+      </x:c>
+      <x:c r="I61" s="16" t="str">
+        <x:v>https://news.google.com/search?q=%E6%9C%88%E4%B9%8B%E6%9A%97%E9%9D%A2%20F%E8%BD%AE%2035%E4%BA%BF%E7%BE%8E%E5%85%83&amp;hl=zh-CN&amp;gl=CN&amp;ceid=CN%3Azh-Hans</x:v>
+      </x:c>
+      <x:c r="J61" s="15" t="n">
+        <x:v>46241.479166666664</x:v>
+      </x:c>
+      <x:c r="K61" s="12" t="str">
+        <x:v>已核验</x:v>
+      </x:c>
+      <x:c r="L61" s="12" t="str">
         <x:v>月之暗面是一家大模型创业公司，推出 Kimi 等面向个人与企业的 AI 产品。其产品以长上下文理解、资料阅读、信息整理和多轮对话为主要能力，覆盖个人效率工具与企业级 AI 应用需求。</x:v>
       </x:c>
-      <x:c r="M47" s="12" t="str">
+      <x:c r="M61" s="12" t="str">
         <x:v>https://www.moonshot.cn/</x:v>
       </x:c>
-      <x:c r="N47" s="12" t="str">
+      <x:c r="N61" s="12" t="str">
         <x:v>产品/售后：support@moonshot.cn；媒体：pr@kimi.com；投资者联系：ir@kimi.com；企业微信客服：微信公众号「月之暗面Kimi」菜单“联系我们”。</x:v>
       </x:c>
     </x:row>
@@ -2694,10 +3284,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="18" t="n">
-        <x:v>46272.42526790509</x:v>
+        <x:v>46272.4316646875</x:v>
       </x:c>
       <x:c r="B2" t="n">
-        <x:v>43</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C2" t="n">
         <x:v>7</x:v>

</xml_diff>